<commit_message>
Regenerate 2026-05-07 ticket eval and related grades artifacts after full grader run.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-07.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-07.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G2" t="n">
-        <v>47.9</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>33.3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>50</v>
+        <v>61.1</v>
       </c>
     </row>
     <row r="10">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="E10" t="n">
         <v>254</v>
       </c>
       <c r="F10" t="n">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="G10" t="n">
-        <v>68.09999999999999</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="E11" t="n">
         <v>179</v>
       </c>
       <c r="F11" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="G11" t="n">
-        <v>72.5</v>
+        <v>70.8</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E12" t="n">
         <v>92</v>
       </c>
       <c r="F12" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G12" t="n">
-        <v>65.2</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="13">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
       </c>
       <c r="F14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G14" t="n">
-        <v>36.1</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E15" t="n">
         <v>6</v>
       </c>
       <c r="F15" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G15" t="n">
-        <v>19.4</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="16">
@@ -874,16 +874,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>19</v>
       </c>
       <c r="F16" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G16" t="n">
-        <v>52.8</v>
+        <v>37.3</v>
       </c>
     </row>
     <row r="17">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>871</v>
+        <v>890</v>
       </c>
       <c r="E17" t="n">
         <v>204</v>
       </c>
       <c r="F17" t="n">
-        <v>667</v>
+        <v>686</v>
       </c>
       <c r="G17" t="n">
-        <v>23.4</v>
+        <v>22.9</v>
       </c>
     </row>
   </sheetData>
@@ -1103,22 +1103,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D2" t="n">
-        <v>64.8</v>
+        <v>63.4</v>
       </c>
       <c r="E2" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F2" t="n">
-        <v>64.2</v>
+        <v>61.8</v>
       </c>
       <c r="G2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H2" t="n">
         <v>64.09999999999999</v>
@@ -1127,34 +1127,34 @@
         <v>92</v>
       </c>
       <c r="J2" t="n">
-        <v>44.4</v>
+        <v>40</v>
       </c>
       <c r="K2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L2" t="n">
-        <v>100</v>
+        <v>33.3</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N2" t="n">
-        <v>50</v>
+        <v>27.3</v>
       </c>
       <c r="O2" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="P2" t="n">
-        <v>36.1</v>
+        <v>35.8</v>
       </c>
       <c r="Q2" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="R2" t="n">
-        <v>61.9</v>
+        <v>46.4</v>
       </c>
       <c r="S2" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -1184,10 +1184,10 @@
         <v>1</v>
       </c>
       <c r="AF2" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="AG2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -1252,22 +1252,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>75.40000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="C4" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D4" t="n">
-        <v>79.09999999999999</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F4" t="n">
-        <v>63.2</v>
+        <v>61.4</v>
       </c>
       <c r="G4" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H4" t="n">
         <v>58</v>
@@ -1276,22 +1276,22 @@
         <v>81</v>
       </c>
       <c r="J4" t="n">
+        <v>40</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" t="n">
         <v>50</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>4</v>
       </c>
-      <c r="L4" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="M4" t="n">
-        <v>3</v>
-      </c>
       <c r="N4" t="n">
-        <v>70.59999999999999</v>
+        <v>54.5</v>
       </c>
       <c r="O4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="P4" t="n">
         <v>32.7</v>
@@ -1300,13 +1300,16 @@
         <v>104</v>
       </c>
       <c r="R4" t="n">
-        <v>39.1</v>
+        <v>35.7</v>
       </c>
       <c r="S4" t="n">
-        <v>23</v>
+        <v>28</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
@@ -1330,10 +1333,10 @@
         <v>1</v>
       </c>
       <c r="AF4" t="n">
-        <v>0</v>
+        <v>55.6</v>
       </c>
       <c r="AG4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1453,22 +1456,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68.09999999999999</v>
+        <v>66</v>
       </c>
       <c r="C7" t="n">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="D7" t="n">
-        <v>72.5</v>
+        <v>70.8</v>
       </c>
       <c r="E7" t="n">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F7" t="n">
-        <v>65.2</v>
+        <v>63.4</v>
       </c>
       <c r="G7" t="n">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="H7" t="n">
         <v>60.2</v>
@@ -1477,40 +1480,40 @@
         <v>181</v>
       </c>
       <c r="J7" t="n">
-        <v>36.1</v>
+        <v>34.2</v>
       </c>
       <c r="K7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L7" t="n">
-        <v>19.4</v>
+        <v>17.6</v>
       </c>
       <c r="M7" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="N7" t="n">
-        <v>52.8</v>
+        <v>37.3</v>
       </c>
       <c r="O7" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="P7" t="n">
-        <v>23.4</v>
+        <v>22.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>871</v>
+        <v>890</v>
       </c>
       <c r="R7" t="n">
-        <v>47.9</v>
+        <v>40</v>
       </c>
       <c r="S7" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="T7" t="n">
-        <v>33.3</v>
+        <v>25</v>
       </c>
       <c r="U7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V7" t="n">
         <v>71.40000000000001</v>
@@ -1540,10 +1543,10 @@
         <v>2</v>
       </c>
       <c r="AF7" t="n">
-        <v>50</v>
+        <v>61.1</v>
       </c>
       <c r="AG7" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>